<commit_message>
docs: add P02 API contract draft
</commit_message>
<xml_diff>
--- a/docs/plan/QuickAssist_KeHoach_PhanCong_GoogleOAuth_CoTen.xlsx
+++ b/docs/plan/QuickAssist_KeHoach_PhanCong_GoogleOAuth_CoTen.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng quan" sheetId="1" r:id="R129ef94f4589476c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ma trận chức năng" sheetId="2" r:id="R682e230181664c06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog phân công" sheetId="3" r:id="Rb7868d59b8e24f8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline 8 tuần" sheetId="4" r:id="R7637aed93646429c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tải công việc" sheetId="5" r:id="R568e231e9722489c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rủi ro &amp; quyết định" sheetId="6" r:id="R119652b44c5c40b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kế hoạch tuần" sheetId="7" r:id="Rd926d4e58e5645c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng quan" sheetId="1" r:id="R67268198bc4647bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ma trận chức năng" sheetId="2" r:id="Rd03c9fac3df041a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog phân công" sheetId="3" r:id="Re781b2c55c314032"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline 8 tuần" sheetId="4" r:id="Rf4acca98c3fe432c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tải công việc" sheetId="5" r:id="R888596cac37447c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rủi ro &amp; quyết định" sheetId="6" r:id="Rd6bd6e519ba44997"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kế hoạch tuần" sheetId="7" r:id="R0827c91433ba4b03"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -458,7 +458,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R687033d5f4724fed"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd9e51e626b76458d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1649,13 +1649,11 @@
           <x:t xml:space="preserve">Không còn endpoint mâu thuẫn; có OAuth flow, request/response/error mẫu</x:t>
         </x:is>
       </x:c>
-      <x:c r="N5" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Chưa bắt đầu</x:t>
-        </x:is>
+      <x:c r="N5" s="3" t="str">
+        <x:v>Chờ duyệt</x:v>
       </x:c>
       <x:c r="O5" s="8" t="n">
-        <x:v>0</x:v>
+        <x:v>0.9</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -6844,7 +6842,7 @@
     <x:mergeCell ref="A1:L1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R145758045a974c7b"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98f127a079ca411e"/>
 </x:worksheet>
 </file>
 

</xml_diff>